<commit_message>
Plan workbook: add Smaregi-ratio monthly sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5mKNMdAhueiuoU89hTodu
</commit_message>
<xml_diff>
--- a/excel/Weekends_予算と報奨金案_粗利2150万円.xlsx
+++ b/excel/Weekends_予算と報奨金案_粗利2150万円.xlsx
@@ -12,7 +12,8 @@
     <sheet name="達成度別" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="粗利率別" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="月別目標と営業利益" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="報奨金（例B）" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="月別（スマレジ版）" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="報奨金（例B）" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -395,6 +396,120 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>月別の営業利益（スマレジ版・100%達成時）</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'月別（スマレジ版）'!G4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'月別（スマレジ版）'!$A$5:$A$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'月別（スマレジ版）'!$G$5:$G$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'月別（スマレジ版）'!H4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'月別（スマレジ版）'!$H$5:$H$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -423,6 +538,33 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -2372,6 +2514,710 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>月別の目標と営業利益　スマレジ版（全月で100%達成した場合）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>月の目標は、店長がスマレジに登録した店舗予算（年6,000万円・税抜）の月比率で配分。前年構成比版との差も表示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>スマレジ予算（参考）</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>月比率</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>目標売上</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>粗利目標100%</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>粗利目標105%</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>営業利益（100%時）</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>累計</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>構成比版との差（粗利目標）</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>実績粗利</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>段階</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>報奨金</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>8月</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="C5" s="10">
+        <f>B5/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D5" s="9">
+        <f>ROUND(入力!$B$19*C5,-3)</f>
+        <v/>
+      </c>
+      <c r="E5" s="9">
+        <f>ROUND(入力!$B$5*C5,-3)</f>
+        <v/>
+      </c>
+      <c r="F5" s="9">
+        <f>ROUND(E5*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G5" s="9">
+        <f>E5-D5*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H5" s="9">
+        <f>SUM($G$5:G5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="9">
+        <f>E5-'月別目標と営業利益'!E5</f>
+        <v/>
+      </c>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="15">
+        <f>IF(J5="","",IF(J5&gt;=F5,2,IF(J5&gt;=E5,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L5" s="9">
+        <f>IF(OR(K5="",K5=0),0,IF(K5=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="C6" s="10">
+        <f>B6/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D6" s="9">
+        <f>ROUND(入力!$B$19*C6,-3)</f>
+        <v/>
+      </c>
+      <c r="E6" s="9">
+        <f>ROUND(入力!$B$5*C6,-3)</f>
+        <v/>
+      </c>
+      <c r="F6" s="9">
+        <f>ROUND(E6*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G6" s="9">
+        <f>E6-D6*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H6" s="9">
+        <f>SUM($G$5:G6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="9">
+        <f>E6-'月別目標と営業利益'!E6</f>
+        <v/>
+      </c>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="15">
+        <f>IF(J6="","",IF(J6&gt;=F6,2,IF(J6&gt;=E6,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L6" s="9">
+        <f>IF(OR(K6="",K6=0),0,IF(K6=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="C7" s="10">
+        <f>B7/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D7" s="9">
+        <f>ROUND(入力!$B$19*C7,-3)</f>
+        <v/>
+      </c>
+      <c r="E7" s="9">
+        <f>ROUND(入力!$B$5*C7,-3)</f>
+        <v/>
+      </c>
+      <c r="F7" s="9">
+        <f>ROUND(E7*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G7" s="9">
+        <f>E7-D7*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H7" s="9">
+        <f>SUM($G$5:G7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="9">
+        <f>E7-'月別目標と営業利益'!E7</f>
+        <v/>
+      </c>
+      <c r="J7" s="4" t="n"/>
+      <c r="K7" s="15">
+        <f>IF(J7="","",IF(J7&gt;=F7,2,IF(J7&gt;=E7,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L7" s="9">
+        <f>IF(OR(K7="",K7=0),0,IF(K7=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="C8" s="10">
+        <f>B8/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D8" s="9">
+        <f>ROUND(入力!$B$19*C8,-3)</f>
+        <v/>
+      </c>
+      <c r="E8" s="9">
+        <f>ROUND(入力!$B$5*C8,-3)</f>
+        <v/>
+      </c>
+      <c r="F8" s="9">
+        <f>ROUND(E8*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G8" s="9">
+        <f>E8-D8*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H8" s="9">
+        <f>SUM($G$5:G8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="9">
+        <f>E8-'月別目標と営業利益'!E8</f>
+        <v/>
+      </c>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="15">
+        <f>IF(J8="","",IF(J8&gt;=F8,2,IF(J8&gt;=E8,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L8" s="9">
+        <f>IF(OR(K8="",K8=0),0,IF(K8=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="C9" s="10">
+        <f>B9/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D9" s="9">
+        <f>ROUND(入力!$B$19*C9,-3)</f>
+        <v/>
+      </c>
+      <c r="E9" s="9">
+        <f>ROUND(入力!$B$5*C9,-3)</f>
+        <v/>
+      </c>
+      <c r="F9" s="9">
+        <f>ROUND(E9*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G9" s="9">
+        <f>E9-D9*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H9" s="9">
+        <f>SUM($G$5:G9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="9">
+        <f>E9-'月別目標と営業利益'!E9</f>
+        <v/>
+      </c>
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="15">
+        <f>IF(J9="","",IF(J9&gt;=F9,2,IF(J9&gt;=E9,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L9" s="9">
+        <f>IF(OR(K9="",K9=0),0,IF(K9=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1月</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="C10" s="10">
+        <f>B10/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D10" s="9">
+        <f>ROUND(入力!$B$19*C10,-3)</f>
+        <v/>
+      </c>
+      <c r="E10" s="9">
+        <f>ROUND(入力!$B$5*C10,-3)</f>
+        <v/>
+      </c>
+      <c r="F10" s="9">
+        <f>ROUND(E10*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G10" s="9">
+        <f>E10-D10*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H10" s="9">
+        <f>SUM($G$5:G10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="9">
+        <f>E10-'月別目標と営業利益'!E10</f>
+        <v/>
+      </c>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="15">
+        <f>IF(J10="","",IF(J10&gt;=F10,2,IF(J10&gt;=E10,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L10" s="9">
+        <f>IF(OR(K10="",K10=0),0,IF(K10=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2月</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="C11" s="10">
+        <f>B11/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D11" s="9">
+        <f>ROUND(入力!$B$19*C11,-3)</f>
+        <v/>
+      </c>
+      <c r="E11" s="9">
+        <f>ROUND(入力!$B$5*C11,-3)</f>
+        <v/>
+      </c>
+      <c r="F11" s="9">
+        <f>ROUND(E11*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G11" s="9">
+        <f>E11-D11*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H11" s="9">
+        <f>SUM($G$5:G11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="9">
+        <f>E11-'月別目標と営業利益'!E11</f>
+        <v/>
+      </c>
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" s="15">
+        <f>IF(J11="","",IF(J11&gt;=F11,2,IF(J11&gt;=E11,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L11" s="9">
+        <f>IF(OR(K11="",K11=0),0,IF(K11=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>3月</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="C12" s="10">
+        <f>B12/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D12" s="9">
+        <f>ROUND(入力!$B$19*C12,-3)</f>
+        <v/>
+      </c>
+      <c r="E12" s="9">
+        <f>ROUND(入力!$B$5*C12,-3)</f>
+        <v/>
+      </c>
+      <c r="F12" s="9">
+        <f>ROUND(E12*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G12" s="9">
+        <f>E12-D12*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H12" s="9">
+        <f>SUM($G$5:G12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="9">
+        <f>E12-'月別目標と営業利益'!E12</f>
+        <v/>
+      </c>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="15">
+        <f>IF(J12="","",IF(J12&gt;=F12,2,IF(J12&gt;=E12,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L12" s="9">
+        <f>IF(OR(K12="",K12=0),0,IF(K12=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="C13" s="10">
+        <f>B13/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D13" s="9">
+        <f>ROUND(入力!$B$19*C13,-3)</f>
+        <v/>
+      </c>
+      <c r="E13" s="9">
+        <f>ROUND(入力!$B$5*C13,-3)</f>
+        <v/>
+      </c>
+      <c r="F13" s="9">
+        <f>ROUND(E13*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G13" s="9">
+        <f>E13-D13*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H13" s="9">
+        <f>SUM($G$5:G13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="9">
+        <f>E13-'月別目標と営業利益'!E13</f>
+        <v/>
+      </c>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="15">
+        <f>IF(J13="","",IF(J13&gt;=F13,2,IF(J13&gt;=E13,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L13" s="9">
+        <f>IF(OR(K13="",K13=0),0,IF(K13=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="C14" s="10">
+        <f>B14/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D14" s="9">
+        <f>ROUND(入力!$B$19*C14,-3)</f>
+        <v/>
+      </c>
+      <c r="E14" s="9">
+        <f>ROUND(入力!$B$5*C14,-3)</f>
+        <v/>
+      </c>
+      <c r="F14" s="9">
+        <f>ROUND(E14*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G14" s="9">
+        <f>E14-D14*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H14" s="9">
+        <f>SUM($G$5:G14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="9">
+        <f>E14-'月別目標と営業利益'!E14</f>
+        <v/>
+      </c>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="15">
+        <f>IF(J14="","",IF(J14&gt;=F14,2,IF(J14&gt;=E14,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L14" s="9">
+        <f>IF(OR(K14="",K14=0),0,IF(K14=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="C15" s="10">
+        <f>B15/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D15" s="9">
+        <f>ROUND(入力!$B$19*C15,-3)</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>ROUND(入力!$B$5*C15,-3)</f>
+        <v/>
+      </c>
+      <c r="F15" s="9">
+        <f>ROUND(E15*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G15" s="9">
+        <f>E15-D15*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H15" s="9">
+        <f>SUM($G$5:G15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="9">
+        <f>E15-'月別目標と営業利益'!E15</f>
+        <v/>
+      </c>
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="15">
+        <f>IF(J15="","",IF(J15&gt;=F15,2,IF(J15&gt;=E15,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L15" s="9">
+        <f>IF(OR(K15="",K15=0),0,IF(K15=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>7月</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="C16" s="10">
+        <f>B16/SUM($B$5:$B$16)</f>
+        <v/>
+      </c>
+      <c r="D16" s="9">
+        <f>ROUND(入力!$B$19*C16,-3)</f>
+        <v/>
+      </c>
+      <c r="E16" s="9">
+        <f>ROUND(入力!$B$5*C16,-3)</f>
+        <v/>
+      </c>
+      <c r="F16" s="9">
+        <f>ROUND(E16*入力!$B$16,-3)</f>
+        <v/>
+      </c>
+      <c r="G16" s="9">
+        <f>E16-D16*入力!$B$9-入力!$B$20/12-入力!$B$14</f>
+        <v/>
+      </c>
+      <c r="H16" s="9">
+        <f>SUM($G$5:G16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="9">
+        <f>E16-'月別目標と営業利益'!E16</f>
+        <v/>
+      </c>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="15">
+        <f>IF(J16="","",IF(J16&gt;=F16,2,IF(J16&gt;=E16,1,0)))</f>
+        <v/>
+      </c>
+      <c r="L16" s="9">
+        <f>IF(OR(K16="",K16=0),0,IF(K16=2,入力!$B$15,入力!$B$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>年計</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>SUM(B5:B16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="14">
+        <f>SUM(D5:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="14">
+        <f>SUM(E5:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="14">
+        <f>SUM(F5:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="14">
+        <f>SUM(G5:G16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="14">
+        <f>SUM(J5:J16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="14">
+        <f>SUM(L5:L16)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>